<commit_message>
Merged regional results from both versions
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/code/modules/tests/python_regional_new_tort_metrics_merged.xlsx
+++ b/code/modules/tests/python_regional_new_tort_metrics_merged.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniwa-my.sharepoint.com/personal/22756463_student_uwa_edu_au/Documents/M4 Backup/dev/octava/code/modules/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="11_54D5686D9559133BDB982411595ED87656CC5A09" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{798A1D31-69D1-1D4D-8EEF-5E132D5980AA}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="11_54D5686D9559133BDB982411595ED87656CC5A09" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8570B77D-F042-0741-881F-0F3437ED0535}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -754,6 +754,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1168,11 +1172,11 @@
         <v>5.1953359436921409E-4</v>
       </c>
       <c r="Q2" s="3">
-        <f t="shared" ref="Q2:S17" si="0">ABS(I2-M2)/M2</f>
+        <f>ABS(I2-M2)/M2</f>
         <v>5.9528128046385721E-2</v>
       </c>
       <c r="R2" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="Q2:S17" si="0">ABS(J2-N2)/N2</f>
         <v>1.5064721596811148E-16</v>
       </c>
       <c r="S2" s="3">

</xml_diff>